<commit_message>
Correct worksheet numbering and valuation assumptions
</commit_message>
<xml_diff>
--- a/model/InterGlobe_Aviation_Equity_Research.xlsx
+++ b/model/InterGlobe_Aviation_Equity_Research.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/keyurmarolia/Documents/PROJECTS/InterGlobe Aviation Equity Research/model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE84362-43F7-B74A-8D04-7372E4BF9D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443B92C9-682E-C249-B9FC-B536F96704C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Cover" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,14 @@
     <sheet name="02_Raw_Financials" sheetId="3" r:id="rId3"/>
     <sheet name="03_Raw_Operating_KPIs" sheetId="4" r:id="rId4"/>
     <sheet name="04_Industry_Data" sheetId="20" r:id="rId5"/>
-    <sheet name="06_Historical_Analysis" sheetId="7" r:id="rId6"/>
-    <sheet name="08_Operating_Model" sheetId="9" r:id="rId7"/>
-    <sheet name="09_Income_Statement" sheetId="10" r:id="rId8"/>
-    <sheet name="10_Balance_Sheet" sheetId="11" r:id="rId9"/>
-    <sheet name="11_Cash_Flow" sheetId="12" r:id="rId10"/>
-    <sheet name="12_Scenarios" sheetId="13" r:id="rId11"/>
-    <sheet name="13_DCF" sheetId="14" r:id="rId12"/>
-    <sheet name="14_Reverse_DCF" sheetId="23" r:id="rId13"/>
+    <sheet name="05_Historical_Analysis" sheetId="7" r:id="rId6"/>
+    <sheet name="06_Operating_Model" sheetId="9" r:id="rId7"/>
+    <sheet name="07_Income_Statement" sheetId="10" r:id="rId8"/>
+    <sheet name="08_Balance_Sheet" sheetId="11" r:id="rId9"/>
+    <sheet name="09_Cash_Flow" sheetId="12" r:id="rId10"/>
+    <sheet name="10_Scenarios" sheetId="13" r:id="rId11"/>
+    <sheet name="11_DCF" sheetId="14" r:id="rId12"/>
+    <sheet name="12_Reverse_DCF" sheetId="23" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -405,7 +405,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1201" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="581">
   <si>
     <t>Purpose</t>
   </si>
@@ -1724,9 +1724,6 @@
     <t>InterGlobe Aviation Limited | INR crore except per-share values</t>
   </si>
   <si>
-    <t>End-of-year discounting and Gordon growth; lease liabilities are treated as debt.</t>
-  </si>
-  <si>
     <t>Forecast Cash Flow</t>
   </si>
   <si>
@@ -1802,9 +1799,6 @@
     <t>Terminal value / enterprise value</t>
   </si>
   <si>
-    <t>Valuation check</t>
-  </si>
-  <si>
     <t>DCF Sensitivity: Value per Share</t>
   </si>
   <si>
@@ -1889,9 +1883,6 @@
     <t>InterGlobe Aviation Limited | Market-implied cash-flow expectations</t>
   </si>
   <si>
-    <t>Shows the uniform cash-flow scaling required for the DCF to match the observed market price.</t>
-  </si>
-  <si>
     <t>Market-Implied Valuation</t>
   </si>
   <si>
@@ -1949,15 +1940,9 @@
     <t>Market Data</t>
   </si>
   <si>
-    <t>Sheets 08 to 10</t>
-  </si>
-  <si>
     <t>A factor below 1.0x indicates lower market-implied cash flow than the base case.</t>
   </si>
   <si>
-    <t>Sheets 11 to 14</t>
-  </si>
-  <si>
     <t>FY2026 Audited Consolidated Results</t>
   </si>
   <si>
@@ -2075,9 +2060,6 @@
     <t>Operating margin</t>
   </si>
   <si>
-    <t>Scenario inputs are analyst assumptions; DCF sensitivity is presented separately on 13_DCF.</t>
-  </si>
-  <si>
     <t>Market price as of</t>
   </si>
   <si>
@@ -2093,9 +2075,6 @@
     <t>Sheets 01 to 04</t>
   </si>
   <si>
-    <t>Sheet 06</t>
-  </si>
-  <si>
     <t>Ex-fuel CASK (including FX)</t>
   </si>
   <si>
@@ -2118,13 +2097,64 @@
   </si>
   <si>
     <t>Independent equity research model; not investment advice.</t>
+  </si>
+  <si>
+    <t>Sheet 05</t>
+  </si>
+  <si>
+    <t>Sheets 06 to 08</t>
+  </si>
+  <si>
+    <t>Sheets 09 to 12</t>
+  </si>
+  <si>
+    <t>FY2027 operating scenarios use analyst assumptions. Valuation sensitivity is on 11_DCF.</t>
+  </si>
+  <si>
+    <t>Operating EBIT excluding other income</t>
+  </si>
+  <si>
+    <t>Asset reinvestment</t>
+  </si>
+  <si>
+    <t>Forecast reinvestment</t>
+  </si>
+  <si>
+    <t>D&amp;A plus change in net PPE and ROU assets; assumes no disposals, impairments or FX revaluations.</t>
+  </si>
+  <si>
+    <t>Historical reinvestment</t>
+  </si>
+  <si>
+    <t>Historical columns show cash capex only; they exclude non-cash lease additions and are not comparable with forecast UFCF.</t>
+  </si>
+  <si>
+    <t>31-Mar-2026 valuation basis. Lease debt and estimated owned/leased asset reinvestment are included.</t>
+  </si>
+  <si>
+    <t>Enterprise value less net debt</t>
+  </si>
+  <si>
+    <t>WACC exceeds terminal growth</t>
+  </si>
+  <si>
+    <t>Other income treatment</t>
+  </si>
+  <si>
+    <t>All other income excluded for valuation; operating compensation is not separately forecast.</t>
+  </si>
+  <si>
+    <t>Scales forecast and terminal UFCF uniformly; September price compared with a March valuation basis.</t>
+  </si>
+  <si>
+    <t>Market price (07-Sep-2026)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="#,##0.0;\(#,##0.0\);\-"/>
     <numFmt numFmtId="165" formatCode="0.00;\(0.00\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);\-"/>
@@ -2136,6 +2166,7 @@
     <numFmt numFmtId="172" formatCode="0.00\x;\(0.00\x\);\-"/>
     <numFmt numFmtId="173" formatCode="#,##0.00;\(#,##0.00\);\-"/>
     <numFmt numFmtId="174" formatCode="#,##0.0"/>
+    <numFmt numFmtId="176" formatCode="#,##0.00;\(#,##0.00\);0.00"/>
   </numFmts>
   <fonts count="42">
     <font>
@@ -2833,7 +2864,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="232">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3283,6 +3314,9 @@
     <xf numFmtId="167" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="170" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="33" fillId="29" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3532,7 +3566,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="28" customHeight="1">
       <c r="A1" s="179" t="s">
-        <v>569</v>
+        <v>562</v>
       </c>
       <c r="B1" s="179"/>
       <c r="C1" s="179"/>
@@ -3550,7 +3584,7 @@
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
       <c r="A2" s="130" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B2" s="130"/>
       <c r="C2" s="130"/>
@@ -3602,7 +3636,7 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="130" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="B5" s="130"/>
       <c r="C5" s="130"/>
@@ -3636,7 +3670,7 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="168" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B7" s="168"/>
       <c r="C7" s="168"/>
@@ -3654,13 +3688,13 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="130" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B8" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C8" s="193">
-        <f>'09_Income_Statement'!E11</f>
+        <f>'07_Income_Statement'!E11</f>
         <v>84961.9</v>
       </c>
       <c r="D8" s="178"/>
@@ -3677,13 +3711,13 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="130" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B9" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="193">
-        <f>'09_Income_Statement'!J11</f>
+        <f>'07_Income_Statement'!J11</f>
         <v>153031.24673536548</v>
       </c>
       <c r="D9" s="178"/>
@@ -3700,13 +3734,13 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="130" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B10" s="130" t="s">
         <v>178</v>
       </c>
       <c r="C10" s="196">
-        <f>'09_Income_Statement'!J25</f>
+        <f>'07_Income_Statement'!J25</f>
         <v>6.2176511787210724E-2</v>
       </c>
       <c r="D10" s="178"/>
@@ -3723,14 +3757,14 @@
     </row>
     <row r="11" spans="1:14" ht="32" customHeight="1">
       <c r="A11" s="130" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B11" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C11" s="193">
-        <f>'11_Cash_Flow'!J16</f>
-        <v>22496.14225907989</v>
+        <f>'09_Cash_Flow'!J16</f>
+        <v>3839.6435862064282</v>
       </c>
       <c r="D11" s="178"/>
       <c r="E11" s="130"/>
@@ -3746,14 +3780,14 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="130" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B12" s="130" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="194">
-        <f>'13_DCF'!C33</f>
-        <v>5534.6635700204497</v>
+      <c r="C12" s="231">
+        <f>'11_DCF'!C33</f>
+        <v>0</v>
       </c>
       <c r="D12" s="195"/>
       <c r="E12" s="130"/>
@@ -3769,13 +3803,13 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="130" t="s">
-        <v>492</v>
+        <v>580</v>
       </c>
       <c r="B13" s="130" t="s">
         <v>46</v>
       </c>
       <c r="C13" s="194">
-        <f>'14_Reverse_DCF'!C7</f>
+        <f>'12_Reverse_DCF'!C7</f>
         <v>5001</v>
       </c>
       <c r="D13" s="195"/>
@@ -3840,7 +3874,7 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="181" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B17" s="181"/>
       <c r="C17" s="181"/>
@@ -3858,7 +3892,7 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="130" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B18" s="130"/>
       <c r="C18" s="130"/>
@@ -3876,7 +3910,7 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="130" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="B19" s="130"/>
       <c r="C19" s="130"/>
@@ -3894,7 +3928,7 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="130" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B20" s="130"/>
       <c r="C20" s="130"/>
@@ -3912,7 +3946,7 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="130" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B21" s="130"/>
       <c r="C21" s="130"/>
@@ -3948,7 +3982,7 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="130" t="s">
-        <v>560</v>
+        <v>554</v>
       </c>
       <c r="B23" s="130"/>
       <c r="C23" s="130"/>
@@ -3998,7 +4032,7 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="181" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B26" s="181"/>
       <c r="C26" s="181"/>
@@ -4016,10 +4050,10 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="130" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B27" s="192" t="s">
-        <v>561</v>
+        <v>555</v>
       </c>
       <c r="C27" s="130"/>
       <c r="D27" s="130"/>
@@ -4036,10 +4070,10 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="130" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B28" s="192" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="C28" s="130"/>
       <c r="D28" s="130"/>
@@ -4056,10 +4090,10 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="130" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B29" s="192" t="s">
-        <v>514</v>
+        <v>565</v>
       </c>
       <c r="C29" s="130"/>
       <c r="D29" s="130"/>
@@ -4076,10 +4110,10 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="130" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B30" s="192" t="s">
-        <v>516</v>
+        <v>566</v>
       </c>
       <c r="C30" s="130"/>
       <c r="D30" s="130"/>
@@ -4112,7 +4146,7 @@
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="181" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B32" s="181"/>
       <c r="C32" s="181"/>
@@ -4133,7 +4167,7 @@
         <v>1</v>
       </c>
       <c r="B33" s="130" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="C33" s="130"/>
       <c r="D33" s="130"/>
@@ -4190,10 +4224,10 @@
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="130" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B36" s="130" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
       <c r="C36" s="130"/>
       <c r="D36" s="130"/>
@@ -4367,42 +4401,42 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="130" t="s">
-        <v>318</v>
+        <v>568</v>
       </c>
       <c r="B9" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="172">
-        <f>'09_Income_Statement'!C24</f>
-        <v>11372.208000000001</v>
+        <f>'07_Income_Statement'!C24-'07_Income_Statement'!C13</f>
+        <v>9045.3870000000006</v>
       </c>
       <c r="D9" s="172">
-        <f>'09_Income_Statement'!D24</f>
-        <v>11551.6</v>
+        <f>'07_Income_Statement'!D24-'07_Income_Statement'!D13</f>
+        <v>8256.2999999999993</v>
       </c>
       <c r="E9" s="172">
-        <f>'09_Income_Statement'!E24</f>
-        <v>2623.7000000000003</v>
+        <f>'07_Income_Statement'!E24-'07_Income_Statement'!E13</f>
+        <v>-1927.7999999999997</v>
       </c>
       <c r="F9" s="172">
-        <f>'09_Income_Statement'!F24</f>
-        <v>4093.7716737603623</v>
+        <f>'07_Income_Statement'!F24-'07_Income_Statement'!F13</f>
+        <v>256.55909536298532</v>
       </c>
       <c r="G9" s="172">
-        <f>'09_Income_Statement'!G24</f>
-        <v>6300.1787742256347</v>
+        <f>'07_Income_Statement'!G24-'07_Income_Statement'!G13</f>
+        <v>2155.9694478464953</v>
       </c>
       <c r="H9" s="172">
-        <f>'09_Income_Statement'!H24</f>
-        <v>7723.9353788641938</v>
+        <f>'07_Income_Statement'!H24-'07_Income_Statement'!H13</f>
+        <v>3394.8502832203521</v>
       </c>
       <c r="I9" s="172">
-        <f>'09_Income_Statement'!I24</f>
-        <v>8858.608980549443</v>
+        <f>'07_Income_Statement'!I24-'07_Income_Statement'!I13</f>
+        <v>4285.2103773272247</v>
       </c>
       <c r="J9" s="172">
-        <f>'09_Income_Statement'!J24</f>
-        <v>9514.9491164530045</v>
+        <f>'07_Income_Statement'!J24-'07_Income_Statement'!J13</f>
+        <v>4924.0117143920406</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -4413,35 +4447,35 @@
         <v>178</v>
       </c>
       <c r="C10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="D10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="E10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="F10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="G10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="H10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="I10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="J10" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
     </row>
@@ -4454,35 +4488,35 @@
       </c>
       <c r="C11" s="172">
         <f>MAX(C9,0)*C10</f>
-        <v>2865.7964160000001</v>
+        <v>2279.4375240000004</v>
       </c>
       <c r="D11" s="172">
         <f>MAX(D9,0)*D10</f>
-        <v>2911.0032000000001</v>
+        <v>2080.5875999999998</v>
       </c>
       <c r="E11" s="172">
         <f>MAX(E9,0)*E10</f>
-        <v>661.17240000000004</v>
+        <v>0</v>
       </c>
       <c r="F11" s="172">
         <f>MAX(F9,0)*F10</f>
-        <v>1031.6304617876112</v>
+        <v>64.652892031472305</v>
       </c>
       <c r="G11" s="172">
         <f>MAX(G9,0)*G10</f>
-        <v>1587.6450511048599</v>
+        <v>543.30430085731678</v>
       </c>
       <c r="H11" s="172">
         <f>MAX(H9,0)*H10</f>
-        <v>1946.4317154737769</v>
+        <v>855.50227137152876</v>
       </c>
       <c r="I11" s="172">
         <f>MAX(I9,0)*I10</f>
-        <v>2232.3694630984596</v>
+        <v>1079.8730150864606</v>
       </c>
       <c r="J11" s="172">
         <f>MAX(J9,0)*J10</f>
-        <v>2397.767177346157</v>
+        <v>1240.8509520267942</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -4494,35 +4528,35 @@
       </c>
       <c r="C12" s="172">
         <f>C9-C11</f>
-        <v>8506.4115840000013</v>
+        <v>6765.9494759999998</v>
       </c>
       <c r="D12" s="172">
         <f>D9-D11</f>
-        <v>8640.5967999999993</v>
+        <v>6175.7123999999994</v>
       </c>
       <c r="E12" s="172">
         <f>E9-E11</f>
-        <v>1962.5276000000003</v>
+        <v>-1927.7999999999997</v>
       </c>
       <c r="F12" s="172">
         <f>F9-F11</f>
-        <v>3062.1412119727511</v>
+        <v>191.90620333151301</v>
       </c>
       <c r="G12" s="172">
         <f>G9-G11</f>
-        <v>4712.533723120775</v>
+        <v>1612.6651469891785</v>
       </c>
       <c r="H12" s="172">
         <f>H9-H11</f>
-        <v>5777.5036633904165</v>
+        <v>2539.3480118488233</v>
       </c>
       <c r="I12" s="172">
         <f>I9-I11</f>
-        <v>6626.2395174509838</v>
+        <v>3205.3373622407644</v>
       </c>
       <c r="J12" s="172">
         <f>J9-J11</f>
-        <v>7117.1819391068475</v>
+        <v>3683.1607623652462</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -4533,76 +4567,76 @@
         <v>26</v>
       </c>
       <c r="C13" s="172">
-        <f>'09_Income_Statement'!C20</f>
+        <f>'07_Income_Statement'!C20</f>
         <v>6425.7290000000003</v>
       </c>
       <c r="D13" s="172">
-        <f>'09_Income_Statement'!D20</f>
+        <f>'07_Income_Statement'!D20</f>
         <v>8680.2000000000007</v>
       </c>
       <c r="E13" s="172">
-        <f>'09_Income_Statement'!E20</f>
+        <f>'07_Income_Statement'!E20</f>
         <v>10808.2</v>
       </c>
       <c r="F13" s="172">
-        <f>'09_Income_Statement'!F20</f>
+        <f>'07_Income_Statement'!F20</f>
         <v>11515.735652571429</v>
       </c>
       <c r="G13" s="172">
-        <f>'09_Income_Statement'!G20</f>
+        <f>'07_Income_Statement'!G20</f>
         <v>12961.159545484801</v>
       </c>
       <c r="H13" s="172">
-        <f>'09_Income_Statement'!H20</f>
+        <f>'07_Income_Statement'!H20</f>
         <v>14624.348973709721</v>
       </c>
       <c r="I13" s="172">
-        <f>'09_Income_Statement'!I20</f>
+        <f>'07_Income_Statement'!I20</f>
         <v>16292.051481146002</v>
       </c>
       <c r="J13" s="172">
-        <f>'09_Income_Statement'!J20</f>
+        <f>'07_Income_Statement'!J20</f>
         <v>17990.806003634472</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="130" t="s">
-        <v>418</v>
+        <v>569</v>
       </c>
       <c r="B14" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C14" s="172">
-        <f>'10_Balance_Sheet'!C67</f>
+        <f>'08_Balance_Sheet'!C67</f>
         <v>1102.645</v>
       </c>
       <c r="D14" s="172">
-        <f>'10_Balance_Sheet'!D67</f>
+        <f>'08_Balance_Sheet'!D67</f>
         <v>1604.8</v>
       </c>
       <c r="E14" s="172">
-        <f>'10_Balance_Sheet'!E67</f>
+        <f>'08_Balance_Sheet'!E67</f>
         <v>2271.8000000000002</v>
       </c>
       <c r="F14" s="172">
-        <f>'10_Balance_Sheet'!F67</f>
-        <v>3357.5610060977051</v>
+        <f>F13+'08_Balance_Sheet'!F35-'08_Balance_Sheet'!E35</f>
+        <v>14552.493652571437</v>
       </c>
       <c r="G14" s="172">
-        <f>'10_Balance_Sheet'!G67</f>
-        <v>4362.3256067148841</v>
+        <f>G13+'08_Balance_Sheet'!G35-'08_Balance_Sheet'!F35</f>
+        <v>15454.527045484792</v>
       </c>
       <c r="H14" s="172">
-        <f>'10_Balance_Sheet'!H67</f>
-        <v>4947.5258235929614</v>
+        <f>H13+'08_Balance_Sheet'!H35-'08_Balance_Sheet'!G35</f>
+        <v>16966.032645709725</v>
       </c>
       <c r="I14" s="172">
-        <f>'10_Balance_Sheet'!I67</f>
-        <v>4850.5742761447773</v>
+        <f>I13+'08_Balance_Sheet'!I35-'08_Balance_Sheet'!H35</f>
+        <v>19060.359109706013</v>
       </c>
       <c r="J14" s="172">
-        <f>'10_Balance_Sheet'!J67</f>
-        <v>5356.0936357377923</v>
+        <f>J13+'08_Balance_Sheet'!J35-'08_Balance_Sheet'!I35</f>
+        <v>20578.571131869656</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" thickBot="1">
@@ -4613,35 +4647,35 @@
         <v>26</v>
       </c>
       <c r="C15" s="172">
-        <f>'10_Balance_Sheet'!C66</f>
+        <f>'08_Balance_Sheet'!C66</f>
         <v>-5349.8310000000019</v>
       </c>
       <c r="D15" s="172">
-        <f>'10_Balance_Sheet'!D66</f>
+        <f>'08_Balance_Sheet'!D66</f>
         <v>-1290.5029999999988</v>
       </c>
       <c r="E15" s="172">
-        <f>'10_Balance_Sheet'!E66</f>
+        <f>'08_Balance_Sheet'!E66</f>
         <v>-1694.1000000000004</v>
       </c>
       <c r="F15" s="172">
-        <f>'10_Balance_Sheet'!F66</f>
+        <f>'08_Balance_Sheet'!F66</f>
         <v>-1904.5113196872117</v>
       </c>
       <c r="G15" s="172">
-        <f>'10_Balance_Sheet'!G66</f>
+        <f>'08_Balance_Sheet'!G66</f>
         <v>-2341.8097327121031</v>
       </c>
       <c r="H15" s="172">
-        <f>'10_Balance_Sheet'!H66</f>
+        <f>'08_Balance_Sheet'!H66</f>
         <v>-2576.214755257075</v>
       </c>
       <c r="I15" s="172">
-        <f>'10_Balance_Sheet'!I66</f>
+        <f>'08_Balance_Sheet'!I66</f>
         <v>-2707.2531199866826</v>
       </c>
       <c r="J15" s="172">
-        <f>'10_Balance_Sheet'!J66</f>
+        <f>'08_Balance_Sheet'!J66</f>
         <v>-2744.2479520763663</v>
       </c>
     </row>
@@ -4654,35 +4688,35 @@
       </c>
       <c r="C16" s="183">
         <f>C12+C13-C14-C15</f>
-        <v>19179.326584000002</v>
+        <v>17438.864476000002</v>
       </c>
       <c r="D16" s="183">
         <f>D12+D13-D14-D15</f>
-        <v>17006.499799999998</v>
+        <v>14541.615400000001</v>
       </c>
       <c r="E16" s="183">
         <f>E12+E13-E14-E15</f>
-        <v>12193.027600000003</v>
+        <v>8302.7000000000007</v>
       </c>
       <c r="F16" s="183">
         <f>F12+F13-F14-F15</f>
-        <v>13124.827178133688</v>
+        <v>-940.34047698128234</v>
       </c>
       <c r="G16" s="183">
         <f>G12+G13-G14-G15</f>
-        <v>15653.177394602797</v>
+        <v>1461.1073797012905</v>
       </c>
       <c r="H16" s="183">
         <f>H12+H13-H14-H15</f>
-        <v>18030.541568764249</v>
+        <v>2773.8790951058945</v>
       </c>
       <c r="I16" s="183">
         <f>I12+I13-I14-I15</f>
-        <v>20774.969842438892</v>
+        <v>3144.2828536674351</v>
       </c>
       <c r="J16" s="183">
         <f>J12+J13-J14-J15</f>
-        <v>22496.14225907989</v>
+        <v>3839.6435862064282</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -4693,42 +4727,46 @@
         <v>178</v>
       </c>
       <c r="C17" s="167">
-        <f>C16/'09_Income_Statement'!C11</f>
-        <v>0.27834714079411715</v>
+        <f>C16/'07_Income_Statement'!C11</f>
+        <v>0.25308803436509125</v>
       </c>
       <c r="D17" s="167">
-        <f>D16/'09_Income_Statement'!D11</f>
-        <v>0.21046892871419218</v>
+        <f>D16/'07_Income_Statement'!D11</f>
+        <v>0.17996402851877843</v>
       </c>
       <c r="E17" s="167">
-        <f>E16/'09_Income_Statement'!E11</f>
-        <v>0.14351171054319647</v>
+        <f>E16/'07_Income_Statement'!E11</f>
+        <v>9.7722626259535178E-2</v>
       </c>
       <c r="F17" s="167">
-        <f>F16/'09_Income_Statement'!F11</f>
-        <v>0.13681626347232825</v>
+        <f>F16/'07_Income_Statement'!F11</f>
+        <v>-9.8023287245036419E-3</v>
       </c>
       <c r="G17" s="167">
-        <f>G16/'09_Income_Statement'!G11</f>
-        <v>0.1435305734217365</v>
+        <f>G16/'07_Income_Statement'!G11</f>
+        <v>1.339750868162819E-2</v>
       </c>
       <c r="H17" s="167">
-        <f>H16/'09_Income_Statement'!H11</f>
-        <v>0.14577420886038123</v>
+        <f>H16/'07_Income_Statement'!H11</f>
+        <v>2.2426394072594977E-2</v>
       </c>
       <c r="I17" s="167">
-        <f>I16/'09_Income_Statement'!I11</f>
-        <v>0.14990471294530455</v>
+        <f>I16/'07_Income_Statement'!I11</f>
+        <v>2.2688014575838553E-2</v>
       </c>
       <c r="J17" s="167">
-        <f>J16/'09_Income_Statement'!J11</f>
-        <v>0.14700358743062528</v>
+        <f>J16/'07_Income_Statement'!J11</f>
+        <v>2.5090585538038928E-2</v>
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="130"/>
+      <c r="A18" s="130" t="s">
+        <v>570</v>
+      </c>
       <c r="B18" s="130"/>
-      <c r="C18" s="172"/>
+      <c r="C18" s="172" t="s">
+        <v>571</v>
+      </c>
       <c r="D18" s="172"/>
       <c r="E18" s="172"/>
       <c r="F18" s="172"/>
@@ -4738,9 +4776,13 @@
       <c r="J18" s="172"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="170"/>
+      <c r="A19" s="170" t="s">
+        <v>572</v>
+      </c>
       <c r="B19" s="170"/>
-      <c r="C19" s="184"/>
+      <c r="C19" s="184" t="s">
+        <v>573</v>
+      </c>
       <c r="D19" s="184"/>
       <c r="E19" s="184"/>
       <c r="F19" s="184"/>
@@ -4750,9 +4792,13 @@
       <c r="J19" s="184"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="130"/>
+      <c r="A20" s="130" t="s">
+        <v>577</v>
+      </c>
       <c r="B20" s="130"/>
-      <c r="C20" s="172"/>
+      <c r="C20" s="172" t="s">
+        <v>578</v>
+      </c>
       <c r="D20" s="172"/>
       <c r="E20" s="172"/>
       <c r="F20" s="172"/>
@@ -4790,7 +4836,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="28" customHeight="1">
       <c r="A1" s="179" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="B1" s="179"/>
       <c r="C1" s="179"/>
@@ -4804,7 +4850,7 @@
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
       <c r="A2" s="130" t="s">
-        <v>548</v>
+        <v>543</v>
       </c>
       <c r="B2" s="130"/>
       <c r="C2" s="130"/>
@@ -4812,7 +4858,7 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="130" t="s">
-        <v>549</v>
+        <v>544</v>
       </c>
       <c r="B3" s="130"/>
       <c r="C3" s="130"/>
@@ -4826,16 +4872,16 @@
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
       <c r="A5" s="215" t="s">
+        <v>466</v>
+      </c>
+      <c r="B5" s="215" t="s">
+        <v>467</v>
+      </c>
+      <c r="C5" s="215" t="s">
         <v>468</v>
       </c>
-      <c r="B5" s="215" t="s">
+      <c r="D5" s="215" t="s">
         <v>469</v>
-      </c>
-      <c r="C5" s="215" t="s">
-        <v>470</v>
-      </c>
-      <c r="D5" s="215" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1">
@@ -4846,13 +4892,13 @@
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
       <c r="A7" s="130" t="s">
-        <v>550</v>
+        <v>545</v>
       </c>
       <c r="B7" s="216">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="C7" s="218">
-        <f>'08_Operating_Model'!F19</f>
+        <f>'06_Operating_Model'!F19</f>
         <v>4.4571428571428484E-2</v>
       </c>
       <c r="D7" s="216">
@@ -4861,13 +4907,13 @@
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1">
       <c r="A8" s="130" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="B8" s="216">
         <v>0.04</v>
       </c>
       <c r="C8" s="212">
-        <f>'08_Operating_Model'!F36</f>
+        <f>'06_Operating_Model'!F36</f>
         <v>8.7719587628866114E-2</v>
       </c>
       <c r="D8" s="216">
@@ -4876,13 +4922,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="130" t="s">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="B9" s="216">
         <v>0.1</v>
       </c>
       <c r="C9" s="212">
-        <f>'08_Operating_Model'!F52</f>
+        <f>'06_Operating_Model'!F52</f>
         <v>0.05</v>
       </c>
       <c r="D9" s="216">
@@ -4891,13 +4937,13 @@
     </row>
     <row r="10" spans="1:10" ht="15" thickBot="1">
       <c r="A10" s="130" t="s">
-        <v>565</v>
+        <v>558</v>
       </c>
       <c r="B10" s="217">
         <v>0.09</v>
       </c>
       <c r="C10" s="212">
-        <f>'08_Operating_Model'!F55</f>
+        <f>'06_Operating_Model'!F55</f>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="D10" s="217">
@@ -4912,35 +4958,35 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="130" t="s">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="B12" s="132">
-        <f>('08_Operating_Model'!$E$18*(1+B$7))*('08_Operating_Model'!$E$35*(1+B$8)+'08_Operating_Model'!$F$37)*100</f>
+        <f>('06_Operating_Model'!$E$18*(1+B$7))*('06_Operating_Model'!$E$35*(1+B$8)+'06_Operating_Model'!$F$37)*100</f>
         <v>90531.84234106529</v>
       </c>
       <c r="C12" s="132">
-        <f>('08_Operating_Model'!$E$18*(1+C$7))*('08_Operating_Model'!$E$35*(1+C$8)+'08_Operating_Model'!$F$37)*100</f>
+        <f>('06_Operating_Model'!$E$18*(1+C$7))*('06_Operating_Model'!$E$35*(1+C$8)+'06_Operating_Model'!$F$37)*100</f>
         <v>95930.314459934423</v>
       </c>
       <c r="D12" s="132">
-        <f>('08_Operating_Model'!$E$18*(1+D$7))*('08_Operating_Model'!$E$35*(1+D$8)+'08_Operating_Model'!$F$37)*100</f>
+        <f>('06_Operating_Model'!$E$18*(1+D$7))*('06_Operating_Model'!$E$35*(1+D$8)+'06_Operating_Model'!$F$37)*100</f>
         <v>100337.47188608247</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="130" t="s">
-        <v>554</v>
+        <v>549</v>
       </c>
       <c r="B13" s="132">
-        <f>('08_Operating_Model'!$E$18*(1+B$7))*('08_Operating_Model'!$E$51*(1+B$9)+'08_Operating_Model'!$E$54*(1+B$10))*100</f>
+        <f>('06_Operating_Model'!$E$18*(1+B$7))*('06_Operating_Model'!$E$51*(1+B$9)+'06_Operating_Model'!$E$54*(1+B$10))*100</f>
         <v>96426.415800000002</v>
       </c>
       <c r="C13" s="132">
-        <f>('08_Operating_Model'!$E$18*(1+C$7))*('08_Operating_Model'!$E$51*(1+C$9)+'08_Operating_Model'!$E$54*(1+C$10))*100</f>
+        <f>('06_Operating_Model'!$E$18*(1+C$7))*('06_Operating_Model'!$E$51*(1+C$9)+'06_Operating_Model'!$E$54*(1+C$10))*100</f>
         <v>95673.755364571422</v>
       </c>
       <c r="D13" s="132">
-        <f>('08_Operating_Model'!$E$18*(1+D$7))*('08_Operating_Model'!$E$51*(1+D$9)+'08_Operating_Model'!$E$54*(1+D$10))*100</f>
+        <f>('06_Operating_Model'!$E$18*(1+D$7))*('06_Operating_Model'!$E$51*(1+D$9)+'06_Operating_Model'!$E$54*(1+D$10))*100</f>
         <v>94900.275600000008</v>
       </c>
     </row>
@@ -4963,7 +5009,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="130" t="s">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="B15" s="219">
         <f>B14/B12</f>
@@ -4980,10 +5026,10 @@
     </row>
     <row r="17" spans="1:4" ht="15">
       <c r="A17" s="214" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B17" s="222" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="C17" s="222"/>
       <c r="D17" s="222"/>
@@ -5031,7 +5077,7 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="130" t="s">
-        <v>439</v>
+        <v>574</v>
       </c>
       <c r="B3" s="130"/>
       <c r="C3" s="130"/>
@@ -5083,7 +5129,7 @@
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
       <c r="A7" s="162" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B7" s="162"/>
       <c r="C7" s="162"/>
@@ -5100,32 +5146,32 @@
         <v>26</v>
       </c>
       <c r="C8" s="172">
-        <f>'11_Cash_Flow'!F16</f>
-        <v>13124.827178133688</v>
+        <f>'09_Cash_Flow'!F16</f>
+        <v>-940.34047698128234</v>
       </c>
       <c r="D8" s="172">
-        <f>'11_Cash_Flow'!G16</f>
-        <v>15653.177394602797</v>
+        <f>'09_Cash_Flow'!G16</f>
+        <v>1461.1073797012905</v>
       </c>
       <c r="E8" s="172">
-        <f>'11_Cash_Flow'!H16</f>
-        <v>18030.541568764249</v>
+        <f>'09_Cash_Flow'!H16</f>
+        <v>2773.8790951058945</v>
       </c>
       <c r="F8" s="172">
-        <f>'11_Cash_Flow'!I16</f>
-        <v>20774.969842438892</v>
+        <f>'09_Cash_Flow'!I16</f>
+        <v>3144.2828536674351</v>
       </c>
       <c r="G8" s="172">
-        <f>'11_Cash_Flow'!J16</f>
-        <v>22496.14225907989</v>
+        <f>'09_Cash_Flow'!J16</f>
+        <v>3839.6435862064282</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="130" t="s">
+        <v>440</v>
+      </c>
+      <c r="B9" s="130" t="s">
         <v>441</v>
-      </c>
-      <c r="B9" s="130" t="s">
-        <v>442</v>
       </c>
       <c r="C9" s="172">
         <v>1</v>
@@ -5145,7 +5191,7 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="130" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B10" s="130" t="s">
         <v>232</v>
@@ -5173,30 +5219,30 @@
     </row>
     <row r="11" spans="1:10" ht="32" customHeight="1">
       <c r="A11" s="130" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B11" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C11" s="172">
         <f>C8*C10</f>
-        <v>11803.24180024397</v>
+        <v>-845.65426071728882</v>
       </c>
       <c r="D11" s="172">
         <f>D8*D10</f>
-        <v>12659.540085745632</v>
+        <v>1181.6736613031028</v>
       </c>
       <c r="E11" s="172">
         <f>E8*E10</f>
-        <v>13113.901077625011</v>
+        <v>2017.4866027057328</v>
       </c>
       <c r="F11" s="172">
         <f>F8*F10</f>
-        <v>13588.491419870777</v>
+        <v>2056.6123995726048</v>
       </c>
       <c r="G11" s="172">
         <f>G8*G10</f>
-        <v>13232.643208562806</v>
+        <v>2258.5487342305923</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -5210,7 +5256,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="162" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B13" s="162"/>
       <c r="C13" s="162"/>
@@ -5221,7 +5267,7 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="130" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B14" s="175">
         <v>6.5000000000000002E-2</v>
@@ -5234,7 +5280,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="130" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B15" s="189">
         <v>1</v>
@@ -5247,7 +5293,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="130" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B16" s="175">
         <v>0.06</v>
@@ -5260,7 +5306,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="130" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B17" s="167">
         <f>B14+B15*B16</f>
@@ -5274,7 +5320,7 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="130" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B18" s="167">
         <v>0.08</v>
@@ -5287,10 +5333,10 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="130" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B19" s="167">
-        <f>'09_Income_Statement'!F36</f>
+        <f>'07_Income_Statement'!F36</f>
         <v>0.252</v>
       </c>
       <c r="C19" s="130"/>
@@ -5301,7 +5347,7 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="130" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B20" s="175">
         <v>0.2</v>
@@ -5314,7 +5360,7 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="130" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B21" s="167">
         <f>B17*(1-B20)+B18*(1-B19)*B20</f>
@@ -5328,7 +5374,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="130" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B22" s="175">
         <v>0.04</v>
@@ -5350,7 +5396,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="162" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B24" s="162"/>
       <c r="C24" s="162"/>
@@ -5361,14 +5407,14 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="130" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B25" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C25" s="190">
         <f>SUM(C11:G11)</f>
-        <v>64397.817592048195</v>
+        <v>6668.6671370947433</v>
       </c>
       <c r="D25" s="130"/>
       <c r="E25" s="130"/>
@@ -5377,14 +5423,14 @@
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="130" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B26" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="190">
         <f>G8</f>
-        <v>22496.14225907989</v>
+        <v>3839.6435862064282</v>
       </c>
       <c r="D26" s="130"/>
       <c r="E26" s="130"/>
@@ -5393,14 +5439,14 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="130" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B27" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C27" s="190">
         <f>C26*(1+B22)/(B21-B22)</f>
-        <v>325088.76096936257</v>
+        <v>55486.17899142237</v>
       </c>
       <c r="D27" s="130"/>
       <c r="E27" s="130"/>
@@ -5409,14 +5455,14 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="130" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B28" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C28" s="190">
         <f>C27/(1+B21)^G9</f>
-        <v>191223.16775379775</v>
+        <v>32637.987488881394</v>
       </c>
       <c r="D28" s="130"/>
       <c r="E28" s="130"/>
@@ -5425,14 +5471,14 @@
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="130" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B29" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C29" s="190">
         <f>C25+C28</f>
-        <v>255620.98534584595</v>
+        <v>39306.654625976138</v>
       </c>
       <c r="D29" s="130"/>
       <c r="E29" s="130"/>
@@ -5441,13 +5487,13 @@
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="130" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="B30" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C30" s="190">
-        <f>'10_Balance_Sheet'!E86</f>
+        <f>'08_Balance_Sheet'!E86</f>
         <v>41532.899999999994</v>
       </c>
       <c r="D30" s="130"/>
@@ -5457,14 +5503,14 @@
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="130" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B31" s="130" t="s">
         <v>26</v>
       </c>
-      <c r="C31" s="190">
-        <f>C29-C30</f>
-        <v>214088.08534584596</v>
+      <c r="C31" s="229">
+        <f>MAX(C29-C30,0)</f>
+        <v>0</v>
       </c>
       <c r="D31" s="130"/>
       <c r="E31" s="130"/>
@@ -5473,13 +5519,13 @@
     </row>
     <row r="32" spans="1:7" ht="15" thickBot="1">
       <c r="A32" s="130" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B32" s="130" t="s">
         <v>329</v>
       </c>
       <c r="C32" s="190">
-        <f>'09_Income_Statement'!E42</f>
+        <f>'07_Income_Statement'!E42</f>
         <v>38.681318681318679</v>
       </c>
       <c r="D32" s="130"/>
@@ -5489,14 +5535,14 @@
     </row>
     <row r="33" spans="1:7" ht="15" thickBot="1">
       <c r="A33" s="130" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B33" s="130" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="188">
+      <c r="C33" s="230">
         <f>C31/C32</f>
-        <v>5534.6635700204497</v>
+        <v>0</v>
       </c>
       <c r="D33" s="130"/>
       <c r="E33" s="130"/>
@@ -5505,14 +5551,14 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="130" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B34" s="130" t="s">
         <v>178</v>
       </c>
       <c r="C34" s="167">
         <f>C28/C29</f>
-        <v>0.74807304061941438</v>
+        <v>0.8303425412172396</v>
       </c>
       <c r="D34" s="130"/>
       <c r="E34" s="130"/>
@@ -5521,7 +5567,7 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="130" t="s">
-        <v>465</v>
+        <v>576</v>
       </c>
       <c r="B35" s="130" t="s">
         <v>259</v>
@@ -5536,9 +5582,16 @@
       <c r="G35" s="130"/>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="130"/>
-      <c r="B36" s="130"/>
-      <c r="C36" s="130"/>
+      <c r="A36" s="130" t="s">
+        <v>575</v>
+      </c>
+      <c r="B36" s="130" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="229">
+        <f>C29-C30</f>
+        <v>-2226.2453740238561</v>
+      </c>
       <c r="D36" s="130"/>
       <c r="E36" s="130"/>
       <c r="F36" s="130"/>
@@ -5555,7 +5608,7 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="162" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B38" s="162"/>
       <c r="C38" s="162"/>
@@ -5567,12 +5620,13 @@
     <row r="39" spans="1:7">
       <c r="A39" s="130"/>
       <c r="B39" s="167" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="C39" s="167">
         <v>0.03</v>
       </c>
       <c r="D39" s="167">
+        <f>$B$22</f>
         <v>0.04</v>
       </c>
       <c r="E39" s="167">
@@ -5587,16 +5641,16 @@
         <v>0.1</v>
       </c>
       <c r="C40" s="190" cm="1">
-        <f t="array" ref="C40">(SUMPRODUCT($C$8:$G$8,1/(1+$B40)^$C$9:$G$9)+($G$8*(1+C$39)/($B40-C$39))/(1+$B40)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>5960.8584664313503</v>
+        <f t="array" ref="C40">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B40)^$C$9:$G$9)+($G$8*(1+C$39)/($B40-C$39))/(1+$B40)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>13.34248057460273</v>
       </c>
       <c r="D40" s="190" cm="1">
-        <f t="array" ref="D40">(SUMPRODUCT($C$8:$G$8,1/(1+$B40)^$C$9:$G$9)+($G$8*(1+D$39)/($B40-D$39))/(1+$B40)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>6906.6311091295429</v>
+        <f t="array" ref="D40">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B40)^$C$9:$G$9)+($G$8*(1+D$39)/($B40-D$39))/(1+$B40)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>174.76704038240277</v>
       </c>
       <c r="E40" s="190" cm="1">
-        <f t="array" ref="E40">(SUMPRODUCT($C$8:$G$8,1/(1+$B40)^$C$9:$G$9)+($G$8*(1+E$39)/($B40-E$39))/(1+$B40)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>8230.7128089070138</v>
+        <f t="array" ref="E40">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B40)^$C$9:$G$9)+($G$8*(1+E$39)/($B40-E$39))/(1+$B40)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>400.76142411332302</v>
       </c>
       <c r="F40" s="130"/>
       <c r="G40" s="130"/>
@@ -5604,19 +5658,20 @@
     <row r="41" spans="1:7">
       <c r="A41" s="130"/>
       <c r="B41" s="167">
-        <v>0.11</v>
+        <f>$B$21</f>
+        <v>0.11196800000000001</v>
       </c>
       <c r="C41" s="190" cm="1">
-        <f t="array" ref="C41">(SUMPRODUCT($C$8:$G$8,1/(1+$B41)^$C$9:$G$9)+($G$8*(1+C$39)/($B41-C$39))/(1+$B41)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>5043.8030354933771</v>
+        <f t="array" ref="C41">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B41)^$C$9:$G$9)+($G$8*(1+C$39)/($B41-C$39))/(1+$B41)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="D41" s="190" cm="1">
-        <f t="array" ref="D41">(SUMPRODUCT($C$8:$G$8,1/(1+$B41)^$C$9:$G$9)+($G$8*(1+D$39)/($B41-D$39))/(1+$B41)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>5727.9144494236552</v>
+        <f t="array" ref="D41">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B41)^$C$9:$G$9)+($G$8*(1+D$39)/($B41-D$39))/(1+$B41)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="E41" s="190" cm="1">
-        <f t="array" ref="E41">(SUMPRODUCT($C$8:$G$8,1/(1+$B41)^$C$9:$G$9)+($G$8*(1+E$39)/($B41-E$39))/(1+$B41)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>6640.0630013306964</v>
+        <f t="array" ref="E41">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B41)^$C$9:$G$9)+($G$8*(1+E$39)/($B41-E$39))/(1+$B41)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>88.030471690110147</v>
       </c>
       <c r="F41" s="130"/>
       <c r="G41" s="130"/>
@@ -5627,16 +5682,16 @@
         <v>0.12</v>
       </c>
       <c r="C42" s="190" cm="1">
-        <f t="array" ref="C42">(SUMPRODUCT($C$8:$G$8,1/(1+$B42)^$C$9:$G$9)+($G$8*(1+C$39)/($B42-C$39))/(1+$B42)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>4331.6321609044435</v>
+        <f t="array" ref="C42">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B42)^$C$9:$G$9)+($G$8*(1+C$39)/($B42-C$39))/(1+$B42)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="D42" s="190" cm="1">
-        <f t="array" ref="D42">(SUMPRODUCT($C$8:$G$8,1/(1+$B42)^$C$9:$G$9)+($G$8*(1+D$39)/($B42-D$39))/(1+$B42)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>4844.9687155529236</v>
+        <f t="array" ref="D42">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B42)^$C$9:$G$9)+($G$8*(1+D$39)/($B42-D$39))/(1+$B42)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="E42" s="190" cm="1">
-        <f t="array" ref="E42">(SUMPRODUCT($C$8:$G$8,1/(1+$B42)^$C$9:$G$9)+($G$8*(1+E$39)/($B42-E$39))/(1+$B42)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>5504.9728572438262</v>
+        <f t="array" ref="E42">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B42)^$C$9:$G$9)+($G$8*(1+E$39)/($B42-E$39))/(1+$B42)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="F42" s="130"/>
       <c r="G42" s="130"/>
@@ -5647,16 +5702,16 @@
         <v>0.13</v>
       </c>
       <c r="C43" s="190" cm="1">
-        <f t="array" ref="C43">(SUMPRODUCT($C$8:$G$8,1/(1+$B43)^$C$9:$G$9)+($G$8*(1+C$39)/($B43-C$39))/(1+$B43)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>3762.8377610374187</v>
+        <f t="array" ref="C43">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B43)^$C$9:$G$9)+($G$8*(1+C$39)/($B43-C$39))/(1+$B43)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="D43" s="190" cm="1">
-        <f t="array" ref="D43">(SUMPRODUCT($C$8:$G$8,1/(1+$B43)^$C$9:$G$9)+($G$8*(1+D$39)/($B43-D$39))/(1+$B43)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>4159.1618729916536</v>
+        <f t="array" ref="D43">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B43)^$C$9:$G$9)+($G$8*(1+D$39)/($B43-D$39))/(1+$B43)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="E43" s="190" cm="1">
-        <f t="array" ref="E43">(SUMPRODUCT($C$8:$G$8,1/(1+$B43)^$C$9:$G$9)+($G$8*(1+E$39)/($B43-E$39))/(1+$B43)^$G$9-'10_Balance_Sheet'!$E$86)/'09_Income_Statement'!$E$42</f>
-        <v>4654.5670129344471</v>
+        <f t="array" ref="E43">MAX((SUMPRODUCT($C$8:$G$8,1/(1+$B43)^$C$9:$G$9)+($G$8*(1+E$39)/($B43-E$39))/(1+$B43)^$G$9-'08_Balance_Sheet'!$E$86)/'07_Income_Statement'!$E$42,0)</f>
+        <v>0</v>
       </c>
       <c r="F43" s="130"/>
       <c r="G43" s="130"/>
@@ -5695,14 +5750,14 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="130" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B2" s="130"/>
       <c r="C2" s="130"/>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="130" t="s">
-        <v>494</v>
+        <v>579</v>
       </c>
       <c r="B3" s="130"/>
       <c r="C3" s="130"/>
@@ -5714,23 +5769,23 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="155" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B5" s="155"/>
       <c r="C5" s="155"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="130" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="B6" s="130"/>
       <c r="C6" s="130" t="s">
-        <v>568</v>
+        <v>561</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="130" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B7" s="130" t="s">
         <v>46</v>
@@ -5741,19 +5796,19 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="130" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B8" s="130" t="s">
         <v>329</v>
       </c>
       <c r="C8" s="176">
-        <f>'09_Income_Statement'!E42</f>
+        <f>'07_Income_Statement'!E42</f>
         <v>38.681318681318679</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="130" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B9" s="130" t="s">
         <v>26</v>
@@ -5771,13 +5826,13 @@
         <v>26</v>
       </c>
       <c r="C10" s="176">
-        <f>'10_Balance_Sheet'!E86</f>
+        <f>'08_Balance_Sheet'!E86</f>
         <v>41532.899999999994</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="130" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="B11" s="130" t="s">
         <v>26</v>
@@ -5789,74 +5844,74 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="130" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B12" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="176">
-        <f>'13_DCF'!C29</f>
-        <v>255620.98534584595</v>
+        <f>'11_DCF'!C29</f>
+        <v>39306.654625976138</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="130" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="B13" s="130" t="s">
         <v>232</v>
       </c>
       <c r="C13" s="187">
         <f>C11/C12</f>
-        <v>0.919244460337862</v>
+        <v>5.9780761543107097</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="130" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="B14" s="130" t="s">
         <v>26</v>
       </c>
       <c r="C14" s="172">
-        <f>'11_Cash_Flow'!J16*C13</f>
-        <v>20679.454150631664</v>
+        <f>'09_Cash_Flow'!J16*C13</f>
+        <v>22953.681763752706</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="130" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B15" s="130" t="s">
         <v>178</v>
       </c>
       <c r="C15" s="167">
-        <f>C14/'09_Income_Statement'!J11</f>
-        <v>0.13513223339539485</v>
+        <f>C14/'07_Income_Statement'!J11</f>
+        <v>0.14999343110264365</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="130" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B16" s="130" t="s">
         <v>178</v>
       </c>
       <c r="C16" s="167">
-        <f>'11_Cash_Flow'!J17</f>
-        <v>0.14700358743062528</v>
+        <f>'09_Cash_Flow'!J17</f>
+        <v>2.5090585538038928E-2</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="130" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="B17" s="130" t="s">
         <v>258</v>
       </c>
       <c r="C17" s="167">
         <f>C15-C16</f>
-        <v>-1.187135403523043E-2</v>
+        <v>0.12490284556460472</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -5871,14 +5926,14 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="155" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="B20" s="155"/>
       <c r="C20" s="155"/>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="130" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B21" s="130"/>
       <c r="C21" s="206">
@@ -5888,24 +5943,24 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="130" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="B22" s="130"/>
       <c r="C22" s="206">
-        <f>'13_DCF'!C33</f>
-        <v>5534.6635700204497</v>
+        <f>'11_DCF'!C33</f>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="130" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="B23" s="130" t="s">
         <v>178</v>
       </c>
       <c r="C23" s="167">
         <f>C22/C21-1</f>
-        <v>0.1067113717297441</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -5915,11 +5970,11 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="155" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="B25" s="155"/>
       <c r="C25" s="155" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
     </row>
   </sheetData>
@@ -6142,7 +6197,7 @@
     </row>
     <row r="17" spans="1:4" ht="15">
       <c r="A17" s="208" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="B17" s="180"/>
       <c r="C17" s="180"/>
@@ -6153,13 +6208,13 @@
         <v>46272</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
     </row>
   </sheetData>
@@ -6326,7 +6381,7 @@
         <v>142</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" customHeight="1">
@@ -11533,7 +11588,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="19">
       <c r="A1" s="179" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="B1" s="179"/>
       <c r="C1" s="179"/>
@@ -11547,7 +11602,7 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="130" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="B2" s="130"/>
       <c r="C2" s="130"/>
@@ -11561,7 +11616,7 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="130" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="B3" s="130"/>
       <c r="C3" s="130"/>
@@ -11593,16 +11648,16 @@
         <v>9</v>
       </c>
       <c r="C5" s="209" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
       <c r="D5" s="209" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="E5" s="209" t="s">
-        <v>529</v>
+        <v>524</v>
       </c>
       <c r="F5" s="209" t="s">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="G5" s="201"/>
       <c r="H5" s="201"/>
@@ -11635,7 +11690,7 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="210" t="s">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="B8" s="210"/>
       <c r="C8" s="210"/>
@@ -11649,7 +11704,7 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="130" t="s">
-        <v>532</v>
+        <v>527</v>
       </c>
       <c r="B9" s="130" t="s">
         <v>180</v>
@@ -11664,7 +11719,7 @@
         <v>420.03</v>
       </c>
       <c r="F9" s="226" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="G9" s="203"/>
       <c r="H9" s="203"/>
@@ -11673,7 +11728,7 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="130" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="B10" s="130" t="s">
         <v>178</v>
@@ -11695,7 +11750,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="130" t="s">
-        <v>535</v>
+        <v>530</v>
       </c>
       <c r="B11" s="130" t="s">
         <v>180</v>
@@ -11710,7 +11765,7 @@
         <v>338.91</v>
       </c>
       <c r="F11" s="167" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="G11" s="191"/>
       <c r="H11" s="191"/>
@@ -11719,7 +11774,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="130" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="B12" s="130" t="s">
         <v>178</v>
@@ -11741,10 +11796,10 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="130" t="s">
-        <v>536</v>
+        <v>531</v>
       </c>
       <c r="B13" s="130" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="C13" s="223">
         <v>2656.43</v>
@@ -11756,7 +11811,7 @@
         <v>2899.5</v>
       </c>
       <c r="F13" s="167" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="G13" s="191"/>
       <c r="H13" s="191"/>
@@ -11765,7 +11820,7 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="130" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="B14" s="130" t="s">
         <v>178</v>
@@ -11799,7 +11854,7 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="211" t="s">
-        <v>538</v>
+        <v>533</v>
       </c>
       <c r="B16" s="211"/>
       <c r="C16" s="211"/>
@@ -11813,7 +11868,7 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="155" t="s">
-        <v>539</v>
+        <v>534</v>
       </c>
       <c r="B17" s="155" t="s">
         <v>178</v>
@@ -11824,7 +11879,7 @@
         <v>0.64200000000000002</v>
       </c>
       <c r="F17" s="162" t="s">
-        <v>540</v>
+        <v>535</v>
       </c>
       <c r="G17" s="155"/>
       <c r="H17" s="155"/>
@@ -11845,7 +11900,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="211" t="s">
-        <v>541</v>
+        <v>536</v>
       </c>
       <c r="B19" s="211"/>
       <c r="C19" s="211"/>
@@ -11859,7 +11914,7 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="130" t="s">
-        <v>542</v>
+        <v>537</v>
       </c>
       <c r="B20" s="130" t="s">
         <v>178</v>
@@ -11867,7 +11922,7 @@
       <c r="C20" s="202"/>
       <c r="D20" s="130"/>
       <c r="E20" s="212">
-        <f>'08_Operating_Model'!F19</f>
+        <f>'06_Operating_Model'!F19</f>
         <v>4.4571428571428484E-2</v>
       </c>
       <c r="F20" s="130"/>
@@ -11878,7 +11933,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="130" t="s">
-        <v>543</v>
+        <v>538</v>
       </c>
       <c r="B21" s="130" t="s">
         <v>178</v>
@@ -11886,7 +11941,7 @@
       <c r="C21" s="202"/>
       <c r="D21" s="130"/>
       <c r="E21" s="212">
-        <f>'08_Operating_Model'!F29</f>
+        <f>'06_Operating_Model'!F29</f>
         <v>3.1409589265259275E-2</v>
       </c>
       <c r="F21" s="130"/>
@@ -11897,11 +11952,11 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="214" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="B22" s="214"/>
       <c r="C22" s="156" t="s">
-        <v>544</v>
+        <v>539</v>
       </c>
       <c r="D22" s="214"/>
       <c r="E22" s="214"/>
@@ -11925,11 +11980,11 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="214" t="s">
-        <v>545</v>
+        <v>540</v>
       </c>
       <c r="B24" s="214"/>
       <c r="C24" s="214" t="s">
-        <v>546</v>
+        <v>541</v>
       </c>
       <c r="D24" s="214"/>
       <c r="E24" s="214"/>
@@ -16322,7 +16377,7 @@
     </row>
     <row r="3" spans="1:10" ht="34" customHeight="1">
       <c r="A3" s="149" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="B3" s="149"/>
       <c r="C3" s="149"/>
@@ -16806,15 +16861,15 @@
         <v>178</v>
       </c>
       <c r="C19" s="68">
-        <f>'06_Historical_Analysis'!K11</f>
+        <f>'05_Historical_Analysis'!K11</f>
         <v>0.21765734265734271</v>
       </c>
       <c r="D19" s="68">
-        <f>'06_Historical_Analysis'!L11</f>
+        <f>'05_Historical_Analysis'!L11</f>
         <v>0.13065326633165819</v>
       </c>
       <c r="E19" s="68">
-        <f>'06_Historical_Analysis'!M11</f>
+        <f>'05_Historical_Analysis'!M11</f>
         <v>9.4603174603174578E-2</v>
       </c>
       <c r="F19" s="65">
@@ -16987,15 +17042,15 @@
         <v>178</v>
       </c>
       <c r="C25" s="68">
-        <f>'06_Historical_Analysis'!K12</f>
+        <f>'05_Historical_Analysis'!K12</f>
         <v>0.27476038338658149</v>
       </c>
       <c r="D25" s="68">
-        <f>'06_Historical_Analysis'!L12</f>
+        <f>'05_Historical_Analysis'!L12</f>
         <v>0.13116123642439437</v>
       </c>
       <c r="E25" s="68">
-        <f>'06_Historical_Analysis'!M12</f>
+        <f>'05_Historical_Analysis'!M12</f>
         <v>7.4593796159527326E-2</v>
       </c>
       <c r="F25" s="65">
@@ -17139,15 +17194,15 @@
         <v>178</v>
       </c>
       <c r="C29" s="68">
-        <f>'06_Historical_Analysis'!K10</f>
+        <f>'05_Historical_Analysis'!K10</f>
         <v>0.24649532710280386</v>
       </c>
       <c r="D29" s="68">
-        <f>'06_Historical_Analysis'!L10</f>
+        <f>'05_Historical_Analysis'!L10</f>
         <v>0.11152764761012168</v>
       </c>
       <c r="E29" s="68">
-        <f>'06_Historical_Analysis'!M10</f>
+        <f>'05_Historical_Analysis'!M10</f>
         <v>4.0472175379426822E-2</v>
       </c>
       <c r="F29" s="65">
@@ -17965,7 +18020,7 @@
     </row>
     <row r="54" spans="1:10" ht="15">
       <c r="A54" s="59" t="s">
-        <v>563</v>
+        <v>556</v>
       </c>
       <c r="B54" s="59" t="s">
         <v>185</v>
@@ -18005,7 +18060,7 @@
     </row>
     <row r="55" spans="1:10" ht="15">
       <c r="A55" s="59" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="B55" s="59" t="s">
         <v>178</v>
@@ -18272,7 +18327,7 @@
     </row>
     <row r="62" spans="1:10" ht="15">
       <c r="A62" s="59" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="B62" s="59" t="s">
         <v>26</v>
@@ -18313,15 +18368,15 @@
         <v>26</v>
       </c>
       <c r="C63" s="67">
-        <f>'06_Historical_Analysis'!K68</f>
+        <f>'05_Historical_Analysis'!K68</f>
         <v>11372.208000000001</v>
       </c>
       <c r="D63" s="67">
-        <f>'06_Historical_Analysis'!L68</f>
+        <f>'05_Historical_Analysis'!L68</f>
         <v>11551.6</v>
       </c>
       <c r="E63" s="67">
-        <f>'06_Historical_Analysis'!M68</f>
+        <f>'05_Historical_Analysis'!M68</f>
         <v>2623.7000000000003</v>
       </c>
       <c r="F63" s="64">
@@ -18505,15 +18560,15 @@
         <v>26</v>
       </c>
       <c r="C68" s="67">
-        <f>'06_Historical_Analysis'!K69</f>
+        <f>'05_Historical_Analysis'!K69</f>
         <v>17797.937000000002</v>
       </c>
       <c r="D68" s="67">
-        <f>'06_Historical_Analysis'!L69</f>
+        <f>'05_Historical_Analysis'!L69</f>
         <v>20231.800000000003</v>
       </c>
       <c r="E68" s="67">
-        <f>'06_Historical_Analysis'!M69</f>
+        <f>'05_Historical_Analysis'!M69</f>
         <v>13431.900000000001</v>
       </c>
       <c r="F68" s="64">
@@ -18697,15 +18752,15 @@
         <v>26</v>
       </c>
       <c r="C73" s="67">
-        <f>'06_Historical_Analysis'!K70</f>
+        <f>'05_Historical_Analysis'!K70</f>
         <v>18873.132000000001</v>
       </c>
       <c r="D73" s="67">
-        <f>'06_Historical_Analysis'!L70</f>
+        <f>'05_Historical_Analysis'!L70</f>
         <v>23242.100000000002</v>
       </c>
       <c r="E73" s="67">
-        <f>'06_Historical_Analysis'!M70</f>
+        <f>'05_Historical_Analysis'!M70</f>
         <v>15516.600000000002</v>
       </c>
       <c r="F73" s="64">
@@ -19385,35 +19440,35 @@
         <v>26</v>
       </c>
       <c r="C9" s="95">
-        <f>'08_Operating_Model'!C39</f>
+        <f>'06_Operating_Model'!C39</f>
         <v>60807.600000000006</v>
       </c>
       <c r="D9" s="95">
-        <f>'08_Operating_Model'!D39</f>
+        <f>'06_Operating_Model'!D39</f>
         <v>69731</v>
       </c>
       <c r="E9" s="95">
-        <f>'08_Operating_Model'!E39</f>
+        <f>'06_Operating_Model'!E39</f>
         <v>73622.999999999985</v>
       </c>
       <c r="F9" s="105">
-        <f>'08_Operating_Model'!F39</f>
+        <f>'06_Operating_Model'!F39</f>
         <v>83650.511758628578</v>
       </c>
       <c r="G9" s="95">
-        <f>'08_Operating_Model'!G39</f>
+        <f>'06_Operating_Model'!G39</f>
         <v>95163.648894192389</v>
       </c>
       <c r="H9" s="95">
-        <f>'08_Operating_Model'!H39</f>
+        <f>'06_Operating_Model'!H39</f>
         <v>108003.07180159677</v>
       </c>
       <c r="I9" s="95">
-        <f>'08_Operating_Model'!I39</f>
+        <f>'06_Operating_Model'!I39</f>
         <v>121018.84281142722</v>
       </c>
       <c r="J9" s="95">
-        <f>'08_Operating_Model'!J39</f>
+        <f>'06_Operating_Model'!J39</f>
         <v>133637.34618223616</v>
       </c>
     </row>
@@ -19425,35 +19480,35 @@
         <v>26</v>
       </c>
       <c r="C10" s="95">
-        <f>'08_Operating_Model'!C40</f>
+        <f>'06_Operating_Model'!C40</f>
         <v>8096.7419999999984</v>
       </c>
       <c r="D10" s="95">
-        <f>'08_Operating_Model'!D40</f>
+        <f>'06_Operating_Model'!D40</f>
         <v>11071.899999999994</v>
       </c>
       <c r="E10" s="95">
-        <f>'08_Operating_Model'!E40</f>
+        <f>'06_Operating_Model'!E40</f>
         <v>11338.900000000009</v>
       </c>
       <c r="F10" s="105">
-        <f>'08_Operating_Model'!F40</f>
+        <f>'06_Operating_Model'!F40</f>
         <v>12279.802701305853</v>
       </c>
       <c r="G10" s="95">
-        <f>'08_Operating_Model'!G40</f>
+        <f>'06_Operating_Model'!G40</f>
         <v>13894.491273679716</v>
       </c>
       <c r="H10" s="95">
-        <f>'08_Operating_Model'!H40</f>
+        <f>'06_Operating_Model'!H40</f>
         <v>15685.073788227262</v>
       </c>
       <c r="I10" s="95">
-        <f>'08_Operating_Model'!I40</f>
+        <f>'06_Operating_Model'!I40</f>
         <v>17568.993649852102</v>
       </c>
       <c r="J10" s="95">
-        <f>'08_Operating_Model'!J40</f>
+        <f>'06_Operating_Model'!J40</f>
         <v>19393.900553129326</v>
       </c>
     </row>
@@ -19465,35 +19520,35 @@
         <v>26</v>
       </c>
       <c r="C11" s="95">
-        <f>'08_Operating_Model'!C43</f>
+        <f>'06_Operating_Model'!C43</f>
         <v>68904.342000000004</v>
       </c>
       <c r="D11" s="95">
-        <f>'08_Operating_Model'!D43</f>
+        <f>'06_Operating_Model'!D43</f>
         <v>80802.899999999994</v>
       </c>
       <c r="E11" s="95">
-        <f>'08_Operating_Model'!E43</f>
+        <f>'06_Operating_Model'!E43</f>
         <v>84961.9</v>
       </c>
       <c r="F11" s="105">
-        <f>'08_Operating_Model'!F43</f>
+        <f>'06_Operating_Model'!F43</f>
         <v>95930.314459934423</v>
       </c>
       <c r="G11" s="95">
-        <f>'08_Operating_Model'!G43</f>
+        <f>'06_Operating_Model'!G43</f>
         <v>109058.1401678721</v>
       </c>
       <c r="H11" s="95">
-        <f>'08_Operating_Model'!H43</f>
+        <f>'06_Operating_Model'!H43</f>
         <v>123688.14558982404</v>
       </c>
       <c r="I11" s="95">
-        <f>'08_Operating_Model'!I43</f>
+        <f>'06_Operating_Model'!I43</f>
         <v>138587.83646127934</v>
       </c>
       <c r="J11" s="95">
-        <f>'08_Operating_Model'!J43</f>
+        <f>'06_Operating_Model'!J43</f>
         <v>153031.24673536548</v>
       </c>
     </row>
@@ -19506,31 +19561,31 @@
       </c>
       <c r="C12" s="96"/>
       <c r="D12" s="96">
-        <f>'08_Operating_Model'!D48</f>
+        <f>'06_Operating_Model'!D48</f>
         <v>0.17268226725102442</v>
       </c>
       <c r="E12" s="96">
-        <f>'08_Operating_Model'!E48</f>
+        <f>'06_Operating_Model'!E48</f>
         <v>5.1470924929674533E-2</v>
       </c>
       <c r="F12" s="106">
-        <f>'08_Operating_Model'!F48</f>
+        <f>'06_Operating_Model'!F48</f>
         <v>0.12909803641319728</v>
       </c>
       <c r="G12" s="96">
-        <f>'08_Operating_Model'!G48</f>
+        <f>'06_Operating_Model'!G48</f>
         <v>0.13684752084723484</v>
       </c>
       <c r="H12" s="96">
-        <f>'08_Operating_Model'!H48</f>
+        <f>'06_Operating_Model'!H48</f>
         <v>0.13414867885544468</v>
       </c>
       <c r="I12" s="96">
-        <f>'08_Operating_Model'!I48</f>
+        <f>'06_Operating_Model'!I48</f>
         <v>0.12046175322949559</v>
       </c>
       <c r="J12" s="96">
-        <f>'08_Operating_Model'!J48</f>
+        <f>'06_Operating_Model'!J48</f>
         <v>0.10421845555054565</v>
       </c>
     </row>
@@ -19542,35 +19597,35 @@
         <v>26</v>
       </c>
       <c r="C13" s="95">
-        <f>'08_Operating_Model'!C60</f>
+        <f>'06_Operating_Model'!C60</f>
         <v>2326.8209999999999</v>
       </c>
       <c r="D13" s="95">
-        <f>'08_Operating_Model'!D60</f>
+        <f>'06_Operating_Model'!D60</f>
         <v>3295.3</v>
       </c>
       <c r="E13" s="95">
-        <f>'08_Operating_Model'!E60</f>
+        <f>'06_Operating_Model'!E60</f>
         <v>4551.5</v>
       </c>
       <c r="F13" s="105">
-        <f>'08_Operating_Model'!F60</f>
+        <f>'06_Operating_Model'!F60</f>
         <v>3837.212578397377</v>
       </c>
       <c r="G13" s="95">
-        <f>'08_Operating_Model'!G60</f>
+        <f>'06_Operating_Model'!G60</f>
         <v>4144.2093263791394</v>
       </c>
       <c r="H13" s="95">
-        <f>'08_Operating_Model'!H60</f>
+        <f>'06_Operating_Model'!H60</f>
         <v>4329.0850956438417</v>
       </c>
       <c r="I13" s="95">
-        <f>'08_Operating_Model'!I60</f>
+        <f>'06_Operating_Model'!I60</f>
         <v>4573.3986032222183</v>
       </c>
       <c r="J13" s="95">
-        <f>'08_Operating_Model'!J60</f>
+        <f>'06_Operating_Model'!J60</f>
         <v>4590.9374020609639</v>
       </c>
     </row>
@@ -19660,23 +19715,23 @@
         <v>25389.200000000001</v>
       </c>
       <c r="F17" s="105">
-        <f>'08_Operating_Model'!F53</f>
+        <f>'06_Operating_Model'!F53</f>
         <v>27846.874560000004</v>
       </c>
       <c r="G17" s="95">
-        <f>'08_Operating_Model'!G53</f>
+        <f>'06_Operating_Model'!G53</f>
         <v>29820.675652992002</v>
       </c>
       <c r="H17" s="95">
-        <f>'08_Operating_Model'!H53</f>
+        <f>'06_Operating_Model'!H53</f>
         <v>33320.622891018567</v>
       </c>
       <c r="I17" s="95">
-        <f>'08_Operating_Model'!I53</f>
+        <f>'06_Operating_Model'!I53</f>
         <v>36939.299012615193</v>
       </c>
       <c r="J17" s="95">
-        <f>'08_Operating_Model'!J53</f>
+        <f>'06_Operating_Model'!J53</f>
         <v>40591.939526361952</v>
       </c>
     </row>
@@ -19700,23 +19755,23 @@
         <v>2084.6999999999998</v>
       </c>
       <c r="F18" s="105">
-        <f>'08_Operating_Model'!F72</f>
+        <f>'06_Operating_Model'!F72</f>
         <v>2068.737154285714</v>
       </c>
       <c r="G18" s="95">
-        <f>'08_Operating_Model'!G72</f>
+        <f>'06_Operating_Model'!G72</f>
         <v>2147.5528711199995</v>
       </c>
       <c r="H18" s="95">
-        <f>'08_Operating_Model'!H72</f>
+        <f>'06_Operating_Model'!H72</f>
         <v>2234.9248811464045</v>
       </c>
       <c r="I18" s="95">
-        <f>'08_Operating_Model'!I72</f>
+        <f>'06_Operating_Model'!I72</f>
         <v>2307.6072898870761</v>
       </c>
       <c r="J18" s="95">
-        <f>'08_Operating_Model'!J72</f>
+        <f>'06_Operating_Model'!J72</f>
         <v>2361.7639484716137</v>
       </c>
     </row>
@@ -19740,23 +19795,23 @@
         <v>45504.6</v>
       </c>
       <c r="F19" s="107">
-        <f>'08_Operating_Model'!F56-F18-F20</f>
+        <f>'06_Operating_Model'!F56-F18-F20</f>
         <v>54242.407997714297</v>
       </c>
       <c r="G19" s="92">
-        <f>'08_Operating_Model'!G56-G18-G20</f>
+        <f>'06_Operating_Model'!G56-G18-G20</f>
         <v>61972.78265042881</v>
       </c>
       <c r="H19" s="92">
-        <f>'08_Operating_Model'!H56-H18-H20</f>
+        <f>'06_Operating_Model'!H56-H18-H20</f>
         <v>70113.398560728994</v>
       </c>
       <c r="I19" s="92">
-        <f>'08_Operating_Model'!I56-I18-I20</f>
+        <f>'06_Operating_Model'!I56-I18-I20</f>
         <v>78763.668300303834</v>
       </c>
       <c r="J19" s="92">
-        <f>'08_Operating_Model'!J56-J18-J20</f>
+        <f>'06_Operating_Model'!J56-J18-J20</f>
         <v>87162.725542505388</v>
       </c>
     </row>
@@ -19780,23 +19835,23 @@
         <v>10808.2</v>
       </c>
       <c r="F20" s="105">
-        <f>'08_Operating_Model'!F67</f>
+        <f>'06_Operating_Model'!F67</f>
         <v>11515.735652571429</v>
       </c>
       <c r="G20" s="95">
-        <f>'08_Operating_Model'!G67</f>
+        <f>'06_Operating_Model'!G67</f>
         <v>12961.159545484801</v>
       </c>
       <c r="H20" s="95">
-        <f>'08_Operating_Model'!H67</f>
+        <f>'06_Operating_Model'!H67</f>
         <v>14624.348973709721</v>
       </c>
       <c r="I20" s="95">
-        <f>'08_Operating_Model'!I67</f>
+        <f>'06_Operating_Model'!I67</f>
         <v>16292.051481146002</v>
       </c>
       <c r="J20" s="95">
-        <f>'08_Operating_Model'!J67</f>
+        <f>'06_Operating_Model'!J67</f>
         <v>17990.806003634472</v>
       </c>
     </row>
@@ -19882,41 +19937,41 @@
     </row>
     <row r="23" spans="1:10" ht="15">
       <c r="A23" s="84" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="B23" s="84" t="s">
         <v>26</v>
       </c>
       <c r="C23" s="92">
-        <f>'08_Operating_Model'!C63-C22</f>
+        <f>'06_Operating_Model'!C63-C22</f>
         <v>-846.45499999999993</v>
       </c>
       <c r="D23" s="92">
-        <f>'08_Operating_Model'!D63-D22</f>
+        <f>'06_Operating_Model'!D63-D22</f>
         <v>-1121.7999999999938</v>
       </c>
       <c r="E23" s="92">
-        <f>'08_Operating_Model'!E63-E22</f>
+        <f>'06_Operating_Model'!E63-E22</f>
         <v>-3102.9999999999968</v>
       </c>
       <c r="F23" s="107">
-        <f>'08_Operating_Model'!F63-F22</f>
+        <f>'06_Operating_Model'!F63-F22</f>
         <v>0</v>
       </c>
       <c r="G23" s="92">
-        <f>'08_Operating_Model'!G63-G22</f>
+        <f>'06_Operating_Model'!G63-G22</f>
         <v>-7.2759576141834259E-12</v>
       </c>
       <c r="H23" s="92">
-        <f>'08_Operating_Model'!H63-H22</f>
+        <f>'06_Operating_Model'!H63-H22</f>
         <v>1.9099388737231493E-11</v>
       </c>
       <c r="I23" s="92">
-        <f>'08_Operating_Model'!I63-I22</f>
+        <f>'06_Operating_Model'!I63-I22</f>
         <v>-2.7284841053187847E-11</v>
       </c>
       <c r="J23" s="92">
-        <f>'08_Operating_Model'!J63-J22</f>
+        <f>'06_Operating_Model'!J63-J22</f>
         <v>0</v>
       </c>
     </row>
@@ -20206,23 +20261,23 @@
         <v>5890.8</v>
       </c>
       <c r="F32" s="107">
-        <f>'10_Balance_Sheet'!F77</f>
+        <f>'08_Balance_Sheet'!F77</f>
         <v>6219.9359999999997</v>
       </c>
       <c r="G32" s="92">
-        <f>'10_Balance_Sheet'!G77</f>
+        <f>'08_Balance_Sheet'!G77</f>
         <v>6020.0110034999998</v>
       </c>
       <c r="H32" s="92">
-        <f>'10_Balance_Sheet'!H77</f>
+        <f>'08_Balance_Sheet'!H77</f>
         <v>5779.7261527950004</v>
       </c>
       <c r="I32" s="92">
-        <f>'10_Balance_Sheet'!I77</f>
+        <f>'08_Balance_Sheet'!I77</f>
         <v>5661.6000114374992</v>
       </c>
       <c r="J32" s="92">
-        <f>'10_Balance_Sheet'!J77</f>
+        <f>'08_Balance_Sheet'!J77</f>
         <v>5689.2306489946877</v>
       </c>
     </row>
@@ -20685,7 +20740,7 @@
     </row>
     <row r="47" spans="1:10" ht="15">
       <c r="A47" s="86" t="s">
-        <v>566</v>
+        <v>559</v>
       </c>
       <c r="B47" s="86"/>
       <c r="C47" s="86"/>
@@ -20842,7 +20897,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="28" customHeight="1" thickBot="1">
       <c r="A1" s="131" t="s">
-        <v>567</v>
+        <v>560</v>
       </c>
       <c r="B1" s="131"/>
       <c r="C1" s="131"/>
@@ -20990,35 +21045,35 @@
         <v>191</v>
       </c>
       <c r="C9" s="134">
-        <f>'08_Operating_Model'!C9</f>
+        <f>'06_Operating_Model'!C9</f>
         <v>304</v>
       </c>
       <c r="D9" s="134">
-        <f>'08_Operating_Model'!D9</f>
+        <f>'06_Operating_Model'!D9</f>
         <v>367</v>
       </c>
       <c r="E9" s="134">
-        <f>'08_Operating_Model'!E9</f>
+        <f>'06_Operating_Model'!E9</f>
         <v>434</v>
       </c>
       <c r="F9" s="134">
-        <f>'08_Operating_Model'!F9</f>
+        <f>'06_Operating_Model'!F9</f>
         <v>441</v>
       </c>
       <c r="G9" s="134">
-        <f>'08_Operating_Model'!G9</f>
+        <f>'06_Operating_Model'!G9</f>
         <v>473</v>
       </c>
       <c r="H9" s="134">
-        <f>'08_Operating_Model'!H9</f>
+        <f>'06_Operating_Model'!H9</f>
         <v>511</v>
       </c>
       <c r="I9" s="134">
-        <f>'08_Operating_Model'!I9</f>
+        <f>'06_Operating_Model'!I9</f>
         <v>551</v>
       </c>
       <c r="J9" s="134">
-        <f>'08_Operating_Model'!J9</f>
+        <f>'06_Operating_Model'!J9</f>
         <v>589</v>
       </c>
     </row>
@@ -21035,23 +21090,23 @@
         <v>72</v>
       </c>
       <c r="F10" s="134">
-        <f>'08_Operating_Model'!F10</f>
+        <f>'06_Operating_Model'!F10</f>
         <v>42</v>
       </c>
       <c r="G10" s="134">
-        <f>'08_Operating_Model'!G10</f>
+        <f>'06_Operating_Model'!G10</f>
         <v>46</v>
       </c>
       <c r="H10" s="134">
-        <f>'08_Operating_Model'!H10</f>
+        <f>'06_Operating_Model'!H10</f>
         <v>48</v>
       </c>
       <c r="I10" s="134">
-        <f>'08_Operating_Model'!I10</f>
+        <f>'06_Operating_Model'!I10</f>
         <v>48</v>
       </c>
       <c r="J10" s="134">
-        <f>'08_Operating_Model'!J10</f>
+        <f>'06_Operating_Model'!J10</f>
         <v>45</v>
       </c>
     </row>
@@ -21068,23 +21123,23 @@
         <v>65</v>
       </c>
       <c r="F11" s="134">
-        <f>'08_Operating_Model'!F11</f>
+        <f>'06_Operating_Model'!F11</f>
         <v>10</v>
       </c>
       <c r="G11" s="134">
-        <f>'08_Operating_Model'!G11</f>
+        <f>'06_Operating_Model'!G11</f>
         <v>8</v>
       </c>
       <c r="H11" s="134">
-        <f>'08_Operating_Model'!H11</f>
+        <f>'06_Operating_Model'!H11</f>
         <v>8</v>
       </c>
       <c r="I11" s="134">
-        <f>'08_Operating_Model'!I11</f>
+        <f>'06_Operating_Model'!I11</f>
         <v>10</v>
       </c>
       <c r="J11" s="134">
-        <f>'08_Operating_Model'!J11</f>
+        <f>'06_Operating_Model'!J11</f>
         <v>10</v>
       </c>
     </row>
@@ -21096,15 +21151,15 @@
         <v>191</v>
       </c>
       <c r="C12" s="134">
-        <f>'08_Operating_Model'!C12</f>
+        <f>'06_Operating_Model'!C12</f>
         <v>63</v>
       </c>
       <c r="D12" s="134">
-        <f>'08_Operating_Model'!D12</f>
+        <f>'06_Operating_Model'!D12</f>
         <v>67</v>
       </c>
       <c r="E12" s="134">
-        <f>'08_Operating_Model'!E12</f>
+        <f>'06_Operating_Model'!E12</f>
         <v>7</v>
       </c>
       <c r="F12" s="134">
@@ -21136,35 +21191,35 @@
         <v>191</v>
       </c>
       <c r="C13" s="134">
-        <f>'08_Operating_Model'!C13</f>
+        <f>'06_Operating_Model'!C13</f>
         <v>367</v>
       </c>
       <c r="D13" s="134">
-        <f>'08_Operating_Model'!D13</f>
+        <f>'06_Operating_Model'!D13</f>
         <v>434</v>
       </c>
       <c r="E13" s="134">
-        <f>'08_Operating_Model'!E13</f>
+        <f>'06_Operating_Model'!E13</f>
         <v>441</v>
       </c>
       <c r="F13" s="134">
-        <f>'08_Operating_Model'!F13</f>
+        <f>'06_Operating_Model'!F13</f>
         <v>473</v>
       </c>
       <c r="G13" s="134">
-        <f>'08_Operating_Model'!G13</f>
+        <f>'06_Operating_Model'!G13</f>
         <v>511</v>
       </c>
       <c r="H13" s="134">
-        <f>'08_Operating_Model'!H13</f>
+        <f>'06_Operating_Model'!H13</f>
         <v>551</v>
       </c>
       <c r="I13" s="134">
-        <f>'08_Operating_Model'!I13</f>
+        <f>'06_Operating_Model'!I13</f>
         <v>589</v>
       </c>
       <c r="J13" s="134">
-        <f>'08_Operating_Model'!J13</f>
+        <f>'06_Operating_Model'!J13</f>
         <v>624</v>
       </c>
     </row>
@@ -21176,35 +21231,35 @@
         <v>178</v>
       </c>
       <c r="C14" s="133">
-        <f>'08_Operating_Model'!C14</f>
+        <f>'06_Operating_Model'!C14</f>
         <v>0.20723684210526305</v>
       </c>
       <c r="D14" s="133">
-        <f>'08_Operating_Model'!D14</f>
+        <f>'06_Operating_Model'!D14</f>
         <v>0.18256130790190728</v>
       </c>
       <c r="E14" s="133">
-        <f>'08_Operating_Model'!E14</f>
+        <f>'06_Operating_Model'!E14</f>
         <v>1.6129032258064502E-2</v>
       </c>
       <c r="F14" s="133">
-        <f>'08_Operating_Model'!F14</f>
+        <f>'06_Operating_Model'!F14</f>
         <v>7.2562358276643923E-2</v>
       </c>
       <c r="G14" s="133">
-        <f>'08_Operating_Model'!G14</f>
+        <f>'06_Operating_Model'!G14</f>
         <v>8.0338266384778034E-2</v>
       </c>
       <c r="H14" s="133">
-        <f>'08_Operating_Model'!H14</f>
+        <f>'06_Operating_Model'!H14</f>
         <v>7.8277886497064575E-2</v>
       </c>
       <c r="I14" s="133">
-        <f>'08_Operating_Model'!I14</f>
+        <f>'06_Operating_Model'!I14</f>
         <v>6.8965517241379226E-2</v>
       </c>
       <c r="J14" s="133">
-        <f>'08_Operating_Model'!J14</f>
+        <f>'06_Operating_Model'!J14</f>
         <v>5.9422750424448223E-2</v>
       </c>
     </row>
@@ -21632,35 +21687,35 @@
         <v>232</v>
       </c>
       <c r="C27" s="135">
-        <f>C20/'08_Operating_Model'!C73</f>
+        <f>C20/'06_Operating_Model'!C73</f>
         <v>2.6168583465637818</v>
       </c>
       <c r="D27" s="135">
-        <f>D20/'08_Operating_Model'!D73</f>
+        <f>D20/'06_Operating_Model'!D73</f>
         <v>2.7970708326700255</v>
       </c>
       <c r="E27" s="135">
-        <f>E20/'08_Operating_Model'!E73</f>
+        <f>E20/'06_Operating_Model'!E73</f>
         <v>4.8943002977456391</v>
       </c>
       <c r="F27" s="135">
-        <f>F20/'08_Operating_Model'!F73</f>
+        <f>F20/'06_Operating_Model'!F73</f>
         <v>4.295839447365041</v>
       </c>
       <c r="G27" s="135">
-        <f>G20/'08_Operating_Model'!G73</f>
+        <f>G20/'06_Operating_Model'!G73</f>
         <v>3.494050945153055</v>
       </c>
       <c r="H27" s="135">
-        <f>H20/'08_Operating_Model'!H73</f>
+        <f>H20/'06_Operating_Model'!H73</f>
         <v>2.9972368315293925</v>
       </c>
       <c r="I27" s="135">
-        <f>I20/'08_Operating_Model'!I73</f>
+        <f>I20/'06_Operating_Model'!I73</f>
         <v>2.6834067181187513</v>
       </c>
       <c r="J27" s="135">
-        <f>J20/'08_Operating_Model'!J73</f>
+        <f>J20/'06_Operating_Model'!J73</f>
         <v>2.4916203111213138</v>
       </c>
     </row>
@@ -21928,35 +21983,35 @@
         <v>26</v>
       </c>
       <c r="C36" s="132">
-        <f>'08_Operating_Model'!C67</f>
+        <f>'06_Operating_Model'!C67</f>
         <v>6425.7290000000003</v>
       </c>
       <c r="D36" s="132">
-        <f>'08_Operating_Model'!D67</f>
+        <f>'06_Operating_Model'!D67</f>
         <v>8680.2000000000007</v>
       </c>
       <c r="E36" s="132">
-        <f>'08_Operating_Model'!E67</f>
+        <f>'06_Operating_Model'!E67</f>
         <v>10808.2</v>
       </c>
       <c r="F36" s="132">
-        <f>'08_Operating_Model'!F67</f>
+        <f>'06_Operating_Model'!F67</f>
         <v>11515.735652571429</v>
       </c>
       <c r="G36" s="132">
-        <f>'08_Operating_Model'!G67</f>
+        <f>'06_Operating_Model'!G67</f>
         <v>12961.159545484801</v>
       </c>
       <c r="H36" s="132">
-        <f>'08_Operating_Model'!H67</f>
+        <f>'06_Operating_Model'!H67</f>
         <v>14624.348973709721</v>
       </c>
       <c r="I36" s="132">
-        <f>'08_Operating_Model'!I67</f>
+        <f>'06_Operating_Model'!I67</f>
         <v>16292.051481146002</v>
       </c>
       <c r="J36" s="132">
-        <f>'08_Operating_Model'!J67</f>
+        <f>'06_Operating_Model'!J67</f>
         <v>17990.806003634472</v>
       </c>
     </row>
@@ -22228,35 +22283,35 @@
         <v>26</v>
       </c>
       <c r="C47" s="132">
-        <f>'08_Operating_Model'!C72</f>
+        <f>'06_Operating_Model'!C72</f>
         <v>1075.1950000000002</v>
       </c>
       <c r="D47" s="132">
-        <f>'08_Operating_Model'!D72</f>
+        <f>'06_Operating_Model'!D72</f>
         <v>3010.3</v>
       </c>
       <c r="E47" s="132">
-        <f>'08_Operating_Model'!E72</f>
+        <f>'06_Operating_Model'!E72</f>
         <v>2084.6999999999998</v>
       </c>
       <c r="F47" s="132">
-        <f>'08_Operating_Model'!F72</f>
+        <f>'06_Operating_Model'!F72</f>
         <v>2068.737154285714</v>
       </c>
       <c r="G47" s="132">
-        <f>'08_Operating_Model'!G72</f>
+        <f>'06_Operating_Model'!G72</f>
         <v>2147.5528711199995</v>
       </c>
       <c r="H47" s="132">
-        <f>'08_Operating_Model'!H72</f>
+        <f>'06_Operating_Model'!H72</f>
         <v>2234.9248811464045</v>
       </c>
       <c r="I47" s="132">
-        <f>'08_Operating_Model'!I72</f>
+        <f>'06_Operating_Model'!I72</f>
         <v>2307.6072898870761</v>
       </c>
       <c r="J47" s="132">
-        <f>'08_Operating_Model'!J72</f>
+        <f>'06_Operating_Model'!J72</f>
         <v>2361.7639484716137</v>
       </c>
     </row>
@@ -22268,35 +22323,35 @@
         <v>185</v>
       </c>
       <c r="C48" s="161">
-        <f>'08_Operating_Model'!C70</f>
+        <f>'06_Operating_Model'!C70</f>
         <v>7.7185570710696344E-2</v>
       </c>
       <c r="D48" s="161">
-        <f>'08_Operating_Model'!D70</f>
+        <f>'06_Operating_Model'!D70</f>
         <v>0.19113015873015876</v>
       </c>
       <c r="E48" s="161">
-        <f>'08_Operating_Model'!E70</f>
+        <f>'06_Operating_Model'!E70</f>
         <v>0.12092227378190254</v>
       </c>
       <c r="F48" s="161">
-        <f>'08_Operating_Model'!F70</f>
+        <f>'06_Operating_Model'!F70</f>
         <v>0.11487616009280741</v>
       </c>
       <c r="G48" s="161">
-        <f>'08_Operating_Model'!G70</f>
+        <f>'06_Operating_Model'!G70</f>
         <v>0.10913235208816703</v>
       </c>
       <c r="H48" s="161">
-        <f>'08_Operating_Model'!H70</f>
+        <f>'06_Operating_Model'!H70</f>
         <v>0.10367573448375868</v>
       </c>
       <c r="I48" s="161">
-        <f>'08_Operating_Model'!I70</f>
+        <f>'06_Operating_Model'!I70</f>
         <v>9.8491947759570736E-2</v>
       </c>
       <c r="J48" s="161">
-        <f>'08_Operating_Model'!J70</f>
+        <f>'06_Operating_Model'!J70</f>
         <v>9.3567350371592195E-2</v>
       </c>
     </row>
@@ -22504,35 +22559,35 @@
         <v>26</v>
       </c>
       <c r="C63" s="176">
-        <f>'09_Income_Statement'!C11</f>
+        <f>'07_Income_Statement'!C11</f>
         <v>68904.342000000004</v>
       </c>
       <c r="D63" s="176">
-        <f>'09_Income_Statement'!D11</f>
+        <f>'07_Income_Statement'!D11</f>
         <v>80802.899999999994</v>
       </c>
       <c r="E63" s="176">
-        <f>'09_Income_Statement'!E11</f>
+        <f>'07_Income_Statement'!E11</f>
         <v>84961.9</v>
       </c>
       <c r="F63" s="176">
-        <f>'09_Income_Statement'!F11</f>
+        <f>'07_Income_Statement'!F11</f>
         <v>95930.314459934423</v>
       </c>
       <c r="G63" s="176">
-        <f>'09_Income_Statement'!G11</f>
+        <f>'07_Income_Statement'!G11</f>
         <v>109058.1401678721</v>
       </c>
       <c r="H63" s="176">
-        <f>'09_Income_Statement'!H11</f>
+        <f>'07_Income_Statement'!H11</f>
         <v>123688.14558982404</v>
       </c>
       <c r="I63" s="176">
-        <f>'09_Income_Statement'!I11</f>
+        <f>'07_Income_Statement'!I11</f>
         <v>138587.83646127934</v>
       </c>
       <c r="J63" s="176">
-        <f>'09_Income_Statement'!J11</f>
+        <f>'07_Income_Statement'!J11</f>
         <v>153031.24673536548</v>
       </c>
     </row>
@@ -22955,15 +23010,15 @@
         <v>178</v>
       </c>
       <c r="C76" s="167">
-        <f>'09_Income_Statement'!C32/C75</f>
+        <f>'07_Income_Statement'!C32/C75</f>
         <v>8.6740256199890828E-2</v>
       </c>
       <c r="D76" s="167">
-        <f>'09_Income_Statement'!D32/D75</f>
+        <f>'07_Income_Statement'!D32/D75</f>
         <v>8.6036205322355466E-2</v>
       </c>
       <c r="E76" s="167">
-        <f>'09_Income_Statement'!E32/E75</f>
+        <f>'07_Income_Statement'!E32/E75</f>
         <v>8.1500287080015776E-2</v>
       </c>
       <c r="F76" s="175">
@@ -22990,15 +23045,15 @@
         <v>26</v>
       </c>
       <c r="C77" s="178">
-        <f>'09_Income_Statement'!C32</f>
+        <f>'07_Income_Statement'!C32</f>
         <v>4169.3540000000003</v>
       </c>
       <c r="D77" s="178">
-        <f>'09_Income_Statement'!D32</f>
+        <f>'07_Income_Statement'!D32</f>
         <v>5080</v>
       </c>
       <c r="E77" s="178">
-        <f>'09_Income_Statement'!E32</f>
+        <f>'07_Income_Statement'!E32</f>
         <v>5890.8</v>
       </c>
       <c r="F77" s="178">
@@ -23162,7 +23217,7 @@
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="130" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="B85" s="130" t="s">
         <v>26</v>
@@ -23180,7 +23235,7 @@
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="130" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="B86" s="130" t="s">
         <v>26</v>
@@ -23203,7 +23258,7 @@
       </c>
       <c r="B87" s="130"/>
       <c r="C87" s="172" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="D87" s="172"/>
       <c r="E87" s="172"/>
@@ -23219,7 +23274,7 @@
       </c>
       <c r="B88" s="130"/>
       <c r="C88" s="172" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="D88" s="172"/>
       <c r="E88" s="172"/>

</xml_diff>

<commit_message>
Standardize workbook theme metadata
</commit_message>
<xml_diff>
--- a/model/InterGlobe_Aviation_Equity_Research.xlsx
+++ b/model/InterGlobe_Aviation_Equity_Research.xlsx
@@ -3339,9 +3339,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3391,7 +3391,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>

<commit_message>
Remove unused workbook add-in metadata
</commit_message>
<xml_diff>
--- a/model/InterGlobe_Aviation_Equity_Research.xlsx
+++ b/model/InterGlobe_Aviation_Equity_Research.xlsx
@@ -3531,28 +3531,6 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{86D29B0B-884D-504B-9A58-CDDFC98E373F}">
-  <we:reference id="wa200010215" version="2.0.0.0" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="wa200010215" version="2.0.0.0" store="en-US" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="bps.codex_control.document_id" value="&quot;de6a964d-85a8-471e-a010-57dade3b591d&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N36"/>

</xml_diff>